<commit_message>
c_rate als constraint den speichern hinzugefügt
</commit_message>
<xml_diff>
--- a/data/b_Optimierung/opt_inst_Leistung.xlsx
+++ b/data/b_Optimierung/opt_inst_Leistung.xlsx
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>322287.67</v>
+        <v>322745.57</v>
       </c>
     </row>
     <row r="3">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>45852.825</v>
+        <v>74515.807</v>
       </c>
     </row>
     <row r="9">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>34830</v>
+        <v>6214</v>
       </c>
     </row>
     <row r="10">
@@ -579,7 +579,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>131144.08</v>
+        <v>173349.98</v>
       </c>
     </row>
   </sheetData>
@@ -610,7 +610,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>525000</v>
+        <v>149031.61</v>
       </c>
     </row>
   </sheetData>
@@ -641,7 +641,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>2650628.4</v>
+        <v>62140</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
anpassungen für vollständige elektrifitierung gemerged mit wärme
</commit_message>
<xml_diff>
--- a/data/b_Optimierung/opt_inst_Leistung.xlsx
+++ b/data/b_Optimierung/opt_inst_Leistung.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,7 +459,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>322745.57</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>365900</v>
+        <v>130576.82</v>
       </c>
     </row>
     <row r="4">
@@ -549,7 +549,7 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>74515.807</v>
+        <v>6528.2254</v>
       </c>
     </row>
     <row r="9">
@@ -564,7 +564,7 @@
         </is>
       </c>
       <c r="C9" t="n">
-        <v>6214</v>
+        <v>8233.5378</v>
       </c>
     </row>
     <row r="10">
@@ -579,7 +579,67 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>173349.98</v>
+        <v>54135.627</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Solarthermie</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>2000000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Tiefengeothermie</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C12" t="n">
+        <v>408</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Flächengeothermie</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C13" t="n">
+        <v>495</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Anderee</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>140739.79</v>
       </c>
     </row>
   </sheetData>
@@ -610,7 +670,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>149031.61</v>
+        <v>13056.451</v>
       </c>
     </row>
   </sheetData>
@@ -641,7 +701,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>62140</v>
+        <v>82335.378</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
mit wandlern -not working
</commit_message>
<xml_diff>
--- a/data/b_Optimierung/opt_inst_Leistung.xlsx
+++ b/data/b_Optimierung/opt_inst_Leistung.xlsx
@@ -10,6 +10,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="inst_leistung" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="batterie_kapazitaet" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="pump_kapazitaet" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="h2_kapazitaet" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Kosten" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -427,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -459,7 +461,7 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1000000</v>
+        <v>83000</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +476,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>365900</v>
+        <v>60976</v>
       </c>
     </row>
     <row r="4">
@@ -489,7 +491,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>81600</v>
+        <v>8473</v>
       </c>
     </row>
     <row r="5">
@@ -504,13 +506,13 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>9439</v>
+        <v>6439</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="inlineStr">
         <is>
-          <t>Geothermie</t>
+          <t>Andere</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -525,7 +527,7 @@
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
-          <t>Andere</t>
+          <t>Batteriespeicher</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -534,13 +536,13 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>50093.925</v>
+        <v>1200</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="inlineStr">
         <is>
-          <t>Batteriespeicher</t>
+          <t>Pumpspeicher</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -549,22 +551,22 @@
         </is>
       </c>
       <c r="C8" t="n">
-        <v>71653.867</v>
+        <v>6214</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="inlineStr">
         <is>
-          <t>Pumpspeicher</t>
+          <t>Wasserstoffkaverne</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Strom</t>
+          <t>Wasserstoff</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>34830</v>
+        <v>547.50791</v>
       </c>
     </row>
     <row r="10">
@@ -579,7 +581,7 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>2000000</v>
+        <v>15700</v>
       </c>
     </row>
     <row r="11">
@@ -624,7 +626,112 @@
         </is>
       </c>
       <c r="C13" t="n">
-        <v>140739.79</v>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Elektrolyseur</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Wasserstoff</t>
+        </is>
+      </c>
+      <c r="C14" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Brennstoffzelle</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="C15" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Verbrennungsmotor</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Strom</t>
+        </is>
+      </c>
+      <c r="C16" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Wasserstoffheizung</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C17" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="1" t="inlineStr">
+        <is>
+          <t>LT-Wärmepumpe</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C18" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="1" t="inlineStr">
+        <is>
+          <t>HT-Wärmepumpe</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="1" t="inlineStr">
+        <is>
+          <t>Stromheizung_direktelektrisch</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Wärme</t>
+        </is>
+      </c>
+      <c r="C20" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -655,7 +762,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>525000</v>
+        <v>2400</v>
       </c>
     </row>
   </sheetData>
@@ -686,7 +793,69 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>3588449.7</v>
+        <v>62140</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Wert</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Wasserstoffkaverne</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>391077.08</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A22:B23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="22">
+      <c r="B22" s="1" t="inlineStr">
+        <is>
+          <t>Annualisierte CAPEX [EUR/Jahr]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="inlineStr">
+        <is>
+          <t>GESAMT</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>82177520.48038934</v>
       </c>
     </row>
   </sheetData>

</xml_diff>